<commit_message>
implements image zoom and small details
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="49">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -85,34 +85,7 @@
     <t xml:space="preserve">meta_funded_by</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Noto Sans Mono"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">&lt;a href="</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Noto Sans Mono"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">https://www.text-plus.org/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Noto Sans Mono"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">"&gt;TEXT+&lt;/a&gt;</t>
-    </r>
+    <t xml:space="preserve">&lt;a href="https://www.text-plus.org/"&gt;TEXT+&lt;/a&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">meta_distributor</t>
@@ -167,6 +140,36 @@
   </si>
   <si>
     <t xml:space="preserve">&lt;a href="https://creativecommons.org/licenses/by/4.0/"&gt;Creative Commons License CC-BY 4.0 (Attribution 4.0 International)&lt;/a&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">language</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprache</t>
+  </si>
+  <si>
+    <t xml:space="preserve">date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">signatories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertragspartner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">locations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Orte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle</t>
   </si>
 </sst>
 </file>
@@ -269,7 +272,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -299,6 +302,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -425,7 +432,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="19" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.57"/>
@@ -434,7 +441,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="4" style="3" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" s="6" customFormat="true" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="6" customFormat="true" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -443,7 +450,7 @@
       </c>
       <c r="C1" s="4"/>
     </row>
-    <row r="2" customFormat="false" ht="38.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -451,7 +458,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -459,7 +466,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -467,7 +474,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -475,7 +482,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -483,7 +490,7 @@
         <v>2023</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="301.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="297" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -491,7 +498,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -499,7 +506,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="235.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="231.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -507,7 +514,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="317.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="313.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -515,15 +522,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="38.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="71.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -531,7 +538,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="71.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>23</v>
       </c>
@@ -539,7 +546,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
@@ -547,7 +554,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="38.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>27</v>
       </c>
@@ -555,7 +562,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
@@ -563,7 +570,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
@@ -571,7 +578,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
         <v>32</v>
       </c>
@@ -579,7 +586,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>33</v>
       </c>
@@ -587,7 +594,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
@@ -595,7 +602,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
@@ -603,7 +610,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="88.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="83.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
@@ -611,9 +618,49 @@
         <v>38</v>
       </c>
     </row>
+    <row r="23" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="19" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B11" r:id="rId1" display="https://www.text-plus.org/"/>
+    <hyperlink ref="B11" r:id="rId1" display="&lt;a href=&quot;https://www.text-plus.org/&quot;&gt;TEXT+&lt;/a&gt;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
implements edition/tranliteration simultaneous rendering
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -218,36 +218,50 @@
     <t xml:space="preserve">imprint_text</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p&gt;Herausgegeben für das Leibniz-Institut für Europäische Geschichte (IEG)&lt;br&gt;
-von Joachim Berger, Irene Dingel und Johannes Paulmann&lt;br&gt;
-Mainz 2016–2023.&lt;br&gt;
-URL: &lt;a href="https://ieg-differences.eu/"&gt;https://ieg-differences.eu&lt;/a&gt;&lt;/p&gt;
-&lt;p&gt;Textredaktion: Joachim Berger&lt;br&gt;
-Normdaten, Verschlagwortung: Ines Grund&lt;br&gt;
-Konzeptionelle Mitarbeit: Sarah Panter&lt;/p&gt;
-&lt;p&gt;Texte der Vorschauartikel, WordPress-Redaktion: Sabine Gruler, Kirsten Wagner&lt;br&gt;
-&lt;a href="http://www.kultourkonzepte.de/"&gt;http://www.kultourkonzepte.de&lt;/a&gt;&lt;/p&gt;
-&lt;p&gt;Übersetzungen: Patrick Baker, Ellen Glebe, Christopher Reid, Niall Williams&lt;/p&gt;
-&lt;p&gt;Datenkuration, Projektleitung Langzeitverfügbarkeit: Fabian Cremer, Thorsten Wübbena&lt;/p&gt;
+    <t xml:space="preserve">&lt;p class="mt-4"&gt;&lt;em&gt;Herausgebende Institution&lt;/em&gt;&lt;/p&gt;
+&lt;p&gt;Leibniz-Institut für Europäische Geschichte (IEG)&lt;br&gt;
+Alte Universitätsstraße 19&lt;br&gt;
+D-55116 Mainz&lt;br&gt;
+&lt;p&gt;Gefördert im Rahmen der 2. Ausschreibungsrunde (2023) „Kooperationsprojekte“ des NFDI-Konsortiums text+ (&lt;a href="https://text-plus.org"&gt;https://text-plus.org&lt;/a&gt;)&lt;/p&gt;
+&lt;p class="mt-4"&gt;&lt;em&gt;Projektteam am IEG&lt;/em&gt;&lt;/p&gt;
+&lt;p&gt;Editorische Verantwortung, Datenbereinigung, -transformation, -anreicherung: Dr. Jaap Geraerts&lt;/p&gt;
+&lt;p&gt;Langzeitverfügbarkeit: Fabian Cremer&lt;/p&gt;
+&lt;p&gt;Projektleitung: Thorsten Wübbena&lt;/p&gt;
 &lt;p class="mt-7"&gt;&lt;strong&gt;Angaben gemäß § 5 TMG&lt;/strong&gt;&lt;/p&gt;
-&lt;p class="mt-4"&gt;&lt;em&gt;Herausgebende Institution&lt;/em&gt;&lt;/p&gt;
+&lt;p class="mt-5"&gt;&lt;em&gt;Verantwortlich für den Inhalt&lt;/em&gt;&lt;/p&gt;
 &lt;p&gt;Leibniz-Institut für Europäische Geschichte (IEG)&lt;br&gt;
 Alte Universitätsstraße 19&lt;br&gt;
 D-55116 Mainz&lt;br&gt;
 &lt;a href="http://www.ieg-mainz.de"&gt;http://www.ieg-mainz.de&lt;/a&gt;
-&lt;a href="mailto:info@ieg-mainz.de"&gt;info@ieg-mainz.de&lt;/a&gt;
+&lt;a href="mailto:info@ieg-mainz.de"&gt;info@ieg-mainz.de&lt;/a&gt;&lt;br /&gt;
 Telefon: ++49 (0) 6131 39 393 50&lt;br&gt;
 Fax: ++ 49 (0) 6131 39 353 26&lt;/p&gt;
-&lt;p class="mt-5"&gt;&lt;em&gt;Verantwortlich für den Inhalt&lt;/em&gt;&lt;/p&gt;
 &lt;p&gt;Prof. Dr. Nicole Reinhardt, Prof. Dr. Johannes Paulmann&lt;/p&gt;
 &lt;p class="mt-5"&gt;&lt;em&gt;Programming and Design&lt;/em&gt;&lt;/p&gt;
 &lt;p&gt;Wendig OÜ&lt;br&gt;
 &lt;a href="https://wendig.io"&gt;https://wendig.io&lt;/a&gt;&lt;/p&gt;
 &lt;p class="mt-5"&gt;&lt;em&gt;Rechtliche Hinweise&lt;/em&gt;&lt;/p&gt;
-&lt;p&gt;„Ortstermine. Umgang mit Differenz in Europa“ wird gemäß deutschem Urheberrecht publiziert, dessen Schutzdauer die international vereinbarte Mindestschutzfrist der Revidierten Berner Übereinkunft (RBÜ) überschreitet und gemäß EU-Recht auf 70 Jahre nach Tod des Urhebers verlängert. Das IEG prüft sorgfältig sämtliche Rechte zur Speicherung und Veröffentlichung von urheberrechtlich geschütztem Material. Urheberrechtlich geschütztes Material, für das keine Rechteklärung erfolgen kann, wird nicht in „Ortstermine“ gespeichert oder veröffentlicht.&lt;/p&gt;
+&lt;p&gt;„Europäische Friedensverträge der Vormoderne in Daten (FriVer+)“ wird gemäß deutschem Urheberrecht publiziert, dessen Schutzdauer die international vereinbarte Mindestschutzfrist der Revidierten Berner Übereinkunft (RBÜ) überschreitet und gemäß EU-Recht auf 70 Jahre nach Tod des Urhebers verlängert. Das IEG prüft sorgfältig sämtliche Rechte zur Speicherung und Veröffentlichung von urheberrechtlich geschütztem Material. Urheberrechtlich geschütztes Material, für das keine Rechteklärung erfolgen kann, wird nicht in „Ortstermine“ gespeichert oder veröffentlicht.&lt;/p&gt;
 &lt;p class="mt-5"&gt;&lt;em&gt;Haftungsausschluss&lt;/em&gt;&lt;/p&gt;
-&lt;p&gt;Trotz sorgfältiger inhaltlicher Kontrolle übernimmt die herausgebende Institution keine Haftung für die Inhalte externer Links. Für den Inhalt der verlinkten Seiten sind ausschließlich deren Betreiber verantwortlich.&lt;/p&gt;
-</t>
+&lt;p&gt;Trotz sorgfältiger inhaltlicher Kontrolle übernimmt die herausgebende Institution keine Haftung für die Inhalte externer Links. Für den Inhalt der verlinkten Seiten sind ausschließlich deren Betreiber verantwortlich.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">privacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datenschutz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">edition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edition</t>
+  </si>
+  <si>
+    <t xml:space="preserve">transliteration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Transkription</t>
   </si>
 </sst>
 </file>
@@ -258,7 +272,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -306,6 +320,13 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Noto Sans Mono"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -356,48 +377,52 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -524,15 +549,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="94.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="53.29"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="119.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="53.33"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="3" width="11.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="83"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="3" width="11.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="6" style="3" width="11.5"/>
   </cols>
   <sheetData>
     <row r="1" s="6" customFormat="true" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -546,7 +571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -578,7 +603,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -605,7 +630,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="773.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="346.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -632,7 +657,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="33.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -640,7 +665,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
@@ -656,7 +681,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="33.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
@@ -733,7 +758,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="83.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="33.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
         <v>48</v>
       </c>
@@ -741,7 +766,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>50</v>
       </c>
@@ -749,7 +774,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>52</v>
       </c>
@@ -757,7 +782,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>54</v>
       </c>
@@ -765,7 +790,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>56</v>
       </c>
@@ -773,7 +798,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>58</v>
       </c>
@@ -781,7 +806,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
         <v>60</v>
       </c>
@@ -789,17 +814,42 @@
         <v>61</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="1035.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="7" t="s">
+      <c r="B29" s="11" t="s">
         <v>63</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B11" r:id="rId1" display="&lt;a href=&quot;https://www.text-plus.org/&quot;&gt;TEXT+&lt;/a&gt;"/>
+    <hyperlink ref="B29" r:id="rId2" display="&lt;p class=&quot;mt-4&quot;&gt;&lt;em&gt;Herausgebende Institution&lt;/em&gt;&lt;/p&gt;&#10;&#10;&lt;p&gt;Leibniz-Institut für Europäische Geschichte (IEG)&lt;br&gt;&#10;Alte Universitätsstraße 19&lt;br&gt;&#10;D-55116 Mainz&lt;br&gt;&#10;&#10;&lt;p&gt;Gefördert im Rahmen der 2. Ausschreibungsrunde (2023) „Kooperationsprojekte“ des NFDI-Konsortiums text+ (&lt;a href=&quot;https://text-plus.org&quot;&gt;https://text-plus.org&lt;/a&gt;)&lt;/p&gt;&#10;&#10;&lt;p class=&quot;mt-4&quot;&gt;&lt;em&gt;Projektteam am IEG&lt;/em&gt;&lt;/p&gt;&#10;&#10;&lt;p&gt;Editorische Verantwortung, Datenbereinigung, -transformation, -anreicherung: Dr. Jaap Geraerts&lt;/p&gt;&#10;&lt;p&gt;Langzeitverfügbarkeit: Fabian Cremer&lt;/p&gt;&#10;&lt;p&gt;Projektleitung: Thorsten Wübbena&lt;/p&gt;&#10;&#10;&#10;&lt;p class=&quot;mt-7&quot;&gt;&lt;strong&gt;Angaben gemäß § 5 TMG&lt;/strong&gt;&lt;/p&gt;&#10;&#10;&lt;p class=&quot;mt-5&quot;&gt;&lt;em&gt;Verantwortlich für den Inhalt&lt;/em&gt;&lt;/p&gt;&#10;&lt;p&gt;Leibniz-Institut für Europäische Geschichte (IEG)&lt;br&gt;&#10;Alte Universitätsstraße 19&lt;br&gt;&#10;D-55116 Mainz&lt;br&gt;&#10;&lt;a href=&quot;http://www.ieg-mainz.de&quot;&gt;http://www.ieg-mainz.de&lt;/a&gt;&#10;&lt;a href=&quot;mailto:info@ieg-mainz.de&quot;&gt;info@ieg-mainz.de&lt;/a&gt;&lt;br /&gt;&#10;Telefon: ++49 (0) 6131 39 393 50&lt;br&gt;&#10;Fax: ++ 49 (0) 6131 39 353 26&lt;/p&gt;&#10;&lt;p&gt;Prof. Dr. Nicole Reinhardt, Prof. Dr. Johannes Paulmann&lt;/p&gt;&#10;&#10;&lt;p class=&quot;mt-5&quot;&gt;&lt;em&gt;Programming and Design&lt;/em&gt;&lt;/p&gt;&#10;&#10;&lt;p&gt;Wendig OÜ&lt;br&gt;&#10;&lt;a href=&quot;https://wendig.io&quot;&gt;https://wendig.io&lt;/a&gt;&lt;/p&gt;&#10;&#10;&lt;p class=&quot;mt-5&quot;&gt;&lt;em&gt;Rechtliche Hinweise&lt;/em&gt;&lt;/p&gt;&#10;&#10;&lt;p&gt;„Europäische Friedensverträge der Vormoderne in Daten (FriVer+)“ wird gemäß deutschem Urheberrecht publiziert, dessen Schutzdauer die international vereinbarte Mindestschutzfrist der Revidierten Berner Übereinkunft (RBÜ) überschreitet und gemäß EU-Recht auf 70 Jahre nach Tod des Urhebers verlängert. Das IEG prüft sorgfältig sämtliche Rechte zur Speicherung und Veröffentlichung von urheberrechtlich geschütztem Material. Urheberrechtlich geschütztes Material, für das keine Rechteklärung erfolgen kann, wird nicht in „Ortstermine“ gespeichert oder veröffentlicht.&lt;/p&gt;&#10;&#10;&lt;p class=&quot;mt-5&quot;&gt;&lt;em&gt;Haftungsausschluss&lt;/em&gt;&lt;/p&gt;&#10;&#10;&lt;p&gt;Trotz sorgfältiger inhaltlicher Kontrolle übernimmt die herausgebende Institution keine Haftung für die Inhalte externer Links. Für den Inhalt der verlinkten Seiten sind ausschließlich deren Betreiber verantwortlich.&lt;/p&gt;"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>

<commit_message>
implements remaining search functionality
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="76">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -263,6 +263,24 @@
   <si>
     <t xml:space="preserve">Transkription</t>
   </si>
+  <si>
+    <t xml:space="preserve">languages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprachen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">show_all</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alle anzeigen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">active_filters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aktive Filter</t>
+  </si>
 </sst>
 </file>
 
@@ -272,7 +290,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -320,13 +338,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF0000FF"/>
-      <name val="Noto Sans Mono"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -377,7 +388,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -419,10 +430,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -549,7 +556,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
@@ -818,7 +825,7 @@
       <c r="A29" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="9" t="s">
         <v>63</v>
       </c>
     </row>
@@ -844,6 +851,30 @@
       </c>
       <c r="B32" s="2" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#16 changes input label
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -292,6 +292,12 @@
   </si>
   <si>
     <t xml:space="preserve">zurück zur Startseite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">search_in_title</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suche im Titel</t>
   </si>
 </sst>
 </file>
@@ -568,7 +574,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
@@ -903,6 +909,14 @@
       </c>
       <c r="B37" s="2" t="s">
         <v>79</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
another fix for #26
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="86">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -298,6 +298,18 @@
   </si>
   <si>
     <t xml:space="preserve">Suche im Titel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">go_to_image</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gehe zu Abbildung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">of</t>
+  </si>
+  <si>
+    <t xml:space="preserve">von</t>
   </si>
 </sst>
 </file>
@@ -574,8 +586,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
-  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C40"/>
+  <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="119.79"/>
@@ -917,6 +929,22 @@
       </c>
       <c r="B38" s="2" t="s">
         <v>81</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more work on #35
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="90">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -310,6 +310,18 @@
   </si>
   <si>
     <t xml:space="preserve">von</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archives</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Archive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">archive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Archiv</t>
   </si>
 </sst>
 </file>
@@ -586,7 +598,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
@@ -945,6 +957,22 @@
       </c>
       <c r="B40" s="2" t="s">
         <v>85</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adds to #37, #39
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="94">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -322,6 +322,18 @@
   </si>
   <si>
     <t xml:space="preserve">Archiv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abstract</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inhalt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drucke</t>
   </si>
 </sst>
 </file>
@@ -598,7 +610,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
@@ -973,6 +985,22 @@
       </c>
       <c r="B42" s="2" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
see #32, #37, #38, #54, #55, #39
</commit_message>
<xml_diff>
--- a/src/translations.xlsx
+++ b/src/translations.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -352,6 +352,12 @@
   </si>
   <si>
     <t xml:space="preserve">Facetten</t>
+  </si>
+  <si>
+    <t xml:space="preserve">biblio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Literatur</t>
   </si>
 </sst>
 </file>
@@ -628,7 +634,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C47"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultColWidth="11.5078125" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="33.52"/>
@@ -1043,6 +1049,14 @@
       </c>
       <c r="B47" s="2" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>